<commit_message>
Ajoute un brief adapté à la ferme pour chaque signal
- Radar 1 : profil de la ferme (18 ha à Douala) et fiche par produit
  (faisable à Douala, projet, délai, prochaine étape, zone de production) ;
  chaque piste du top reçoit « À retenir », « Que faire » et un verdict
  « Pour ta ferme », avec les prix en FCFA
- Top 15 plus utile : 4 marchés hors d'Afrique au plus, produits sans
  action possible écartés ; 5 tentatives par requête Comtrade
- Radar 2 : projets de la ferme en premier, brief par appel d'offres et
  par actualité, produits en français, nom du journal retiré du titre
- Modèle Google Sheets et guide mis à jour

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017BSHrzMi5jWYWQb6aVx3o3
</commit_message>
<xml_diff>
--- a/signaux-afrique/modele-google-sheets.xlsx
+++ b/signaux-afrique/modele-google-sheets.xlsx
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S1"/>
+  <dimension ref="A1:U1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -449,6 +449,8 @@
     <col width="16" customWidth="1" min="17" max="17"/>
     <col width="48" customWidth="1" min="18" max="18"/>
     <col width="48" customWidth="1" min="19" max="19"/>
+    <col width="16" customWidth="1" min="20" max="20"/>
+    <col width="48" customWidth="1" min="21" max="21"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -544,7 +546,17 @@
       </c>
       <c r="S1" s="1" t="inlineStr">
         <is>
-          <t>resume</t>
+          <t>a_retenir</t>
+        </is>
+      </c>
+      <c r="T1" s="1" t="inlineStr">
+        <is>
+          <t>pour_ma_ferme</t>
+        </is>
+      </c>
+      <c r="U1" s="1" t="inlineStr">
+        <is>
+          <t>que_faire</t>
         </is>
       </c>
     </row>
@@ -559,7 +571,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O1"/>
+  <dimension ref="A1:R1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -568,15 +580,18 @@
     <col width="16" customWidth="1" min="4" max="4"/>
     <col width="16" customWidth="1" min="5" max="5"/>
     <col width="16" customWidth="1" min="6" max="6"/>
-    <col width="48" customWidth="1" min="7" max="7"/>
-    <col width="16" customWidth="1" min="8" max="8"/>
-    <col width="16" customWidth="1" min="9" max="9"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="48" customWidth="1" min="8" max="8"/>
+    <col width="48" customWidth="1" min="9" max="9"/>
     <col width="48" customWidth="1" min="10" max="10"/>
     <col width="16" customWidth="1" min="11" max="11"/>
     <col width="16" customWidth="1" min="12" max="12"/>
-    <col width="16" customWidth="1" min="13" max="13"/>
-    <col width="48" customWidth="1" min="14" max="14"/>
+    <col width="48" customWidth="1" min="13" max="13"/>
+    <col width="16" customWidth="1" min="14" max="14"/>
     <col width="16" customWidth="1" min="15" max="15"/>
+    <col width="16" customWidth="1" min="16" max="16"/>
+    <col width="48" customWidth="1" min="17" max="17"/>
+    <col width="16" customWidth="1" min="18" max="18"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -592,65 +607,80 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
+          <t>concerne_projet</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
           <t>type</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>source</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>pays</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>produits</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>titre</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>a_retenir</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>que_faire</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>lien</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>acheteur</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>contact</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>date_limite</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>date</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>statut</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>notes</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>id</t>
         </is>
@@ -658,7 +688,7 @@
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation sqref="M2:M5000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="P2:P5000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"nouveau,à creuser,contacté,en discussion,deal,sans suite"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>